<commit_message>
BWI sync — 2026-09-14 15:39 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Mexico.xlsx
+++ b/BWI/bestwine_output/bestwine_Mexico.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA486"/>
+  <dimension ref="A1:AA525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -51296,6 +51296,3061 @@
         </is>
       </c>
     </row>
+    <row r="487">
+      <c r="A487" s="2" t="inlineStr">
+        <is>
+          <t>A&amp;B Wines</t>
+        </is>
+      </c>
+      <c r="B487" s="2" t="inlineStr"/>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>168625</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E487" s="2" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G487" s="2" t="inlineStr">
+        <is>
+          <t>Acatempan 2068</t>
+        </is>
+      </c>
+      <c r="H487" s="2" t="inlineStr">
+        <is>
+          <t>44619</t>
+        </is>
+      </c>
+      <c r="I487" s="2" t="inlineStr">
+        <is>
+          <t>https://abwines.mx</t>
+        </is>
+      </c>
+      <c r="J487" s="2" t="inlineStr"/>
+      <c r="K487" s="2" t="inlineStr"/>
+      <c r="L487" s="2" t="inlineStr"/>
+      <c r="M487" s="2" t="inlineStr"/>
+      <c r="N487" s="2" t="inlineStr">
+        <is>
+          <t>info@abwines.mx</t>
+        </is>
+      </c>
+      <c r="O487" s="2" t="inlineStr">
+        <is>
+          <t>+52 33 2005 0675</t>
+        </is>
+      </c>
+      <c r="P487" s="2" t="inlineStr"/>
+      <c r="Q487" s="2" t="inlineStr"/>
+      <c r="R487" s="2" t="inlineStr"/>
+      <c r="S487" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/aybwines/</t>
+        </is>
+      </c>
+      <c r="T487" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/abwines_mx/</t>
+        </is>
+      </c>
+      <c r="U487" s="2" t="inlineStr"/>
+      <c r="V487" s="2" t="inlineStr"/>
+      <c r="W487" s="2" t="inlineStr"/>
+      <c r="X487" s="2" t="inlineStr"/>
+      <c r="Y487" s="2" t="inlineStr"/>
+      <c r="Z487" s="2" t="inlineStr"/>
+      <c r="AA487" s="2" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>Bodegas el Pamplonica S.A. De C.V.</t>
+        </is>
+      </c>
+      <c r="B488" s="2" t="inlineStr"/>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>168624</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E488" s="2" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+      <c r="F488" s="2" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+      <c r="G488" s="2" t="inlineStr">
+        <is>
+          <t>Martín Alonso Pinzon, 848. Fraccionamiento Reforma</t>
+        </is>
+      </c>
+      <c r="H488" s="2" t="inlineStr">
+        <is>
+          <t>91919</t>
+        </is>
+      </c>
+      <c r="I488" s="2" t="inlineStr">
+        <is>
+          <t>https://bodegaselpamplonica.com</t>
+        </is>
+      </c>
+      <c r="J488" s="2" t="inlineStr"/>
+      <c r="K488" s="2" t="inlineStr"/>
+      <c r="L488" s="2" t="inlineStr"/>
+      <c r="M488" s="2" t="inlineStr"/>
+      <c r="N488" s="2" t="inlineStr">
+        <is>
+          <t>bodegaselpamplonica@gmail.com</t>
+        </is>
+      </c>
+      <c r="O488" s="2" t="inlineStr">
+        <is>
+          <t>+52 229 935 0057</t>
+        </is>
+      </c>
+      <c r="P488" s="2" t="inlineStr"/>
+      <c r="Q488" s="2" t="inlineStr"/>
+      <c r="R488" s="2" t="inlineStr"/>
+      <c r="S488" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/pinordenmexico</t>
+        </is>
+      </c>
+      <c r="T488" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/pinordenmexico/</t>
+        </is>
+      </c>
+      <c r="U488" s="2" t="inlineStr"/>
+      <c r="V488" s="2" t="inlineStr"/>
+      <c r="W488" s="2" t="inlineStr"/>
+      <c r="X488" s="2" t="inlineStr"/>
+      <c r="Y488" s="2" t="inlineStr"/>
+      <c r="Z488" s="2" t="inlineStr"/>
+      <c r="AA488" s="2" t="inlineStr"/>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Wine</t>
+        </is>
+      </c>
+      <c r="B489" s="2" t="inlineStr"/>
+      <c r="C489" s="2" t="inlineStr">
+        <is>
+          <t>168623</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E489" s="2" t="inlineStr">
+        <is>
+          <t>Playa del Carmen</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="inlineStr">
+        <is>
+          <t>Quintana Roo</t>
+        </is>
+      </c>
+      <c r="G489" s="2" t="inlineStr">
+        <is>
+          <t>Avenida 75 N Mza</t>
+        </is>
+      </c>
+      <c r="H489" s="2" t="inlineStr">
+        <is>
+          <t>77712</t>
+        </is>
+      </c>
+      <c r="I489" s="2" t="inlineStr">
+        <is>
+          <t>https://drwine.com.mx</t>
+        </is>
+      </c>
+      <c r="J489" s="2" t="inlineStr"/>
+      <c r="K489" s="2" t="inlineStr"/>
+      <c r="L489" s="2" t="inlineStr"/>
+      <c r="M489" s="2" t="inlineStr"/>
+      <c r="N489" s="2" t="inlineStr">
+        <is>
+          <t>info@drwine.com.mx</t>
+        </is>
+      </c>
+      <c r="O489" s="2" t="inlineStr"/>
+      <c r="P489" s="2" t="inlineStr"/>
+      <c r="Q489" s="2" t="inlineStr"/>
+      <c r="R489" s="2" t="inlineStr"/>
+      <c r="S489" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Dr-Wine-110103141329292/</t>
+        </is>
+      </c>
+      <c r="T489" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/drwine.store/</t>
+        </is>
+      </c>
+      <c r="U489" s="2" t="inlineStr"/>
+      <c r="V489" s="2" t="inlineStr"/>
+      <c r="W489" s="2" t="inlineStr"/>
+      <c r="X489" s="2" t="inlineStr"/>
+      <c r="Y489" s="2" t="inlineStr"/>
+      <c r="Z489" s="2" t="inlineStr"/>
+      <c r="AA489" s="2" t="inlineStr"/>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>Hipervinos</t>
+        </is>
+      </c>
+      <c r="B490" s="2" t="inlineStr"/>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>168622</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E490" s="2" t="inlineStr">
+        <is>
+          <t>Zapopan</t>
+        </is>
+      </c>
+      <c r="F490" s="2" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G490" s="2" t="inlineStr">
+        <is>
+          <t>Calz. Circunvalación Oriente 288</t>
+        </is>
+      </c>
+      <c r="H490" s="2" t="inlineStr"/>
+      <c r="I490" s="2" t="inlineStr">
+        <is>
+          <t>https://hipervinos.mx</t>
+        </is>
+      </c>
+      <c r="J490" s="2" t="inlineStr"/>
+      <c r="K490" s="2" t="inlineStr"/>
+      <c r="L490" s="2" t="inlineStr"/>
+      <c r="M490" s="2" t="inlineStr"/>
+      <c r="N490" s="2" t="inlineStr">
+        <is>
+          <t>ventas@hipervinos.mx</t>
+        </is>
+      </c>
+      <c r="O490" s="2" t="inlineStr"/>
+      <c r="P490" s="2" t="inlineStr"/>
+      <c r="Q490" s="2" t="inlineStr"/>
+      <c r="R490" s="2" t="inlineStr"/>
+      <c r="S490" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/hipervinosmx</t>
+        </is>
+      </c>
+      <c r="T490" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/hipervinos</t>
+        </is>
+      </c>
+      <c r="U490" s="2" t="inlineStr"/>
+      <c r="V490" s="2" t="inlineStr"/>
+      <c r="W490" s="2" t="inlineStr">
+        <is>
+          <t>Tania Priscilla Sahagun</t>
+        </is>
+      </c>
+      <c r="X490" s="2" t="inlineStr">
+        <is>
+          <t>Sales Executive</t>
+        </is>
+      </c>
+      <c r="Y490" s="2" t="inlineStr"/>
+      <c r="Z490" s="2" t="inlineStr"/>
+      <c r="AA490" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/tania-priscilla-sahagun-616848148</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="inlineStr">
+        <is>
+          <t>Hipervinos</t>
+        </is>
+      </c>
+      <c r="B491" s="2" t="inlineStr"/>
+      <c r="C491" s="2" t="inlineStr">
+        <is>
+          <t>168622</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E491" s="2" t="inlineStr">
+        <is>
+          <t>Zapopan</t>
+        </is>
+      </c>
+      <c r="F491" s="2" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G491" s="2" t="inlineStr">
+        <is>
+          <t>Calz. Circunvalación Oriente 288</t>
+        </is>
+      </c>
+      <c r="H491" s="2" t="inlineStr"/>
+      <c r="I491" s="2" t="inlineStr">
+        <is>
+          <t>https://hipervinos.mx</t>
+        </is>
+      </c>
+      <c r="J491" s="2" t="inlineStr"/>
+      <c r="K491" s="2" t="inlineStr"/>
+      <c r="L491" s="2" t="inlineStr"/>
+      <c r="M491" s="2" t="inlineStr"/>
+      <c r="N491" s="2" t="inlineStr">
+        <is>
+          <t>ventas@hipervinos.mx</t>
+        </is>
+      </c>
+      <c r="O491" s="2" t="inlineStr"/>
+      <c r="P491" s="2" t="inlineStr"/>
+      <c r="Q491" s="2" t="inlineStr"/>
+      <c r="R491" s="2" t="inlineStr"/>
+      <c r="S491" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/hipervinosmx</t>
+        </is>
+      </c>
+      <c r="T491" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/hipervinos</t>
+        </is>
+      </c>
+      <c r="U491" s="2" t="inlineStr"/>
+      <c r="V491" s="2" t="inlineStr"/>
+      <c r="W491" s="2" t="inlineStr">
+        <is>
+          <t>Oscar Eduardo Dominguez</t>
+        </is>
+      </c>
+      <c r="X491" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wine Business Manager </t>
+        </is>
+      </c>
+      <c r="Y491" s="2" t="inlineStr"/>
+      <c r="Z491" s="2" t="inlineStr"/>
+      <c r="AA491" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/oscar-eduardo-dom%c3%adnguez-8387967a</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>Importadora Reina del Plata</t>
+        </is>
+      </c>
+      <c r="B492" s="2" t="inlineStr"/>
+      <c r="C492" s="2" t="inlineStr">
+        <is>
+          <t>168621</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E492" s="2" t="inlineStr">
+        <is>
+          <t>Zapopan</t>
+        </is>
+      </c>
+      <c r="F492" s="2" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G492" s="2" t="inlineStr">
+        <is>
+          <t>Av. Aviación 5180 L. 1 Plaza Palma Real</t>
+        </is>
+      </c>
+      <c r="H492" s="2" t="inlineStr">
+        <is>
+          <t>45019</t>
+        </is>
+      </c>
+      <c r="I492" s="2" t="inlineStr">
+        <is>
+          <t>https://importadorareinadelplata.com</t>
+        </is>
+      </c>
+      <c r="J492" s="2" t="inlineStr"/>
+      <c r="K492" s="2" t="inlineStr"/>
+      <c r="L492" s="2" t="inlineStr"/>
+      <c r="M492" s="2" t="inlineStr"/>
+      <c r="N492" s="2" t="inlineStr">
+        <is>
+          <t>corporativo@importadorareinadelplata.com</t>
+        </is>
+      </c>
+      <c r="O492" s="2" t="inlineStr"/>
+      <c r="P492" s="2" t="inlineStr"/>
+      <c r="Q492" s="2" t="inlineStr"/>
+      <c r="R492" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/importadora-reina-del-plata</t>
+        </is>
+      </c>
+      <c r="S492" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100094663584620</t>
+        </is>
+      </c>
+      <c r="T492" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/importadorareinadelplata</t>
+        </is>
+      </c>
+      <c r="U492" s="2" t="inlineStr"/>
+      <c r="V492" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@ReinaDelPlataImportadora</t>
+        </is>
+      </c>
+      <c r="W492" s="2" t="inlineStr">
+        <is>
+          <t>Mariana Ferrero</t>
+        </is>
+      </c>
+      <c r="X492" s="2" t="inlineStr">
+        <is>
+          <t>Founding Partner and Executive Director</t>
+        </is>
+      </c>
+      <c r="Y492" s="2" t="inlineStr"/>
+      <c r="Z492" s="2" t="inlineStr"/>
+      <c r="AA492" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mariana-ferrero-5612b1105/</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="inlineStr">
+        <is>
+          <t>Luana Consorcio</t>
+        </is>
+      </c>
+      <c r="B493" s="2" t="inlineStr"/>
+      <c r="C493" s="2" t="inlineStr">
+        <is>
+          <t>168619</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E493" s="2" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+      <c r="F493" s="2" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+      <c r="G493" s="2" t="inlineStr">
+        <is>
+          <t>Av. Miguel Alemán 2577 Col. Adolfo López Mateos</t>
+        </is>
+      </c>
+      <c r="H493" s="2" t="inlineStr"/>
+      <c r="I493" s="2" t="inlineStr">
+        <is>
+          <t>https://consorcioluana.com.mx</t>
+        </is>
+      </c>
+      <c r="J493" s="2" t="inlineStr"/>
+      <c r="K493" s="2" t="inlineStr"/>
+      <c r="L493" s="2" t="inlineStr"/>
+      <c r="M493" s="2" t="inlineStr"/>
+      <c r="N493" s="2" t="inlineStr">
+        <is>
+          <t>recepcion@consorcioluana.com</t>
+        </is>
+      </c>
+      <c r="O493" s="2" t="inlineStr"/>
+      <c r="P493" s="2" t="inlineStr"/>
+      <c r="Q493" s="2" t="inlineStr"/>
+      <c r="R493" s="2" t="inlineStr"/>
+      <c r="S493" s="2" t="inlineStr"/>
+      <c r="T493" s="2" t="inlineStr"/>
+      <c r="U493" s="2" t="inlineStr"/>
+      <c r="V493" s="2" t="inlineStr"/>
+      <c r="W493" s="2" t="inlineStr"/>
+      <c r="X493" s="2" t="inlineStr"/>
+      <c r="Y493" s="2" t="inlineStr"/>
+      <c r="Z493" s="2" t="inlineStr"/>
+      <c r="AA493" s="2" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>La Cava de Baco</t>
+        </is>
+      </c>
+      <c r="B494" s="2" t="inlineStr"/>
+      <c r="C494" s="2" t="inlineStr">
+        <is>
+          <t>168615</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E494" s="2" t="inlineStr">
+        <is>
+          <t>Santiago de Querétaro</t>
+        </is>
+      </c>
+      <c r="F494" s="2" t="inlineStr">
+        <is>
+          <t>Querétaro</t>
+        </is>
+      </c>
+      <c r="G494" s="2" t="inlineStr">
+        <is>
+          <t>Av. Peñuelas 5</t>
+        </is>
+      </c>
+      <c r="H494" s="2" t="inlineStr">
+        <is>
+          <t>76148</t>
+        </is>
+      </c>
+      <c r="I494" s="2" t="inlineStr">
+        <is>
+          <t>https://lacavadebaco.com.mx</t>
+        </is>
+      </c>
+      <c r="J494" s="2" t="inlineStr"/>
+      <c r="K494" s="2" t="inlineStr"/>
+      <c r="L494" s="2" t="inlineStr"/>
+      <c r="M494" s="2" t="inlineStr"/>
+      <c r="N494" s="2" t="inlineStr">
+        <is>
+          <t>marketing@lacavadebaco.com.mx</t>
+        </is>
+      </c>
+      <c r="O494" s="2" t="inlineStr"/>
+      <c r="P494" s="2" t="inlineStr"/>
+      <c r="Q494" s="2" t="inlineStr"/>
+      <c r="R494" s="2" t="inlineStr"/>
+      <c r="S494" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/lacavadebacoqro</t>
+        </is>
+      </c>
+      <c r="T494" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/la_cava_de_baco?fbclid=IwY2xjawSC8uNleHRuA2FlbQIxMABicmlkETFVSGNtSFpxTmpjUFFZT05Hc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHk_gsGrJk-tbmpDwlq9mhrzJmG1MjE6w7yODB7kYXE7n3TZ3Gm1ZsoSXhiwS_aem_1N2ZNW5K7nTaF6WsE0K3qQ</t>
+        </is>
+      </c>
+      <c r="U494" s="2" t="inlineStr"/>
+      <c r="V494" s="2" t="inlineStr"/>
+      <c r="W494" s="2" t="inlineStr">
+        <is>
+          <t>Cecilia Becerra Becerra</t>
+        </is>
+      </c>
+      <c r="X494" s="2" t="inlineStr">
+        <is>
+          <t>Sales Representative</t>
+        </is>
+      </c>
+      <c r="Y494" s="2" t="inlineStr"/>
+      <c r="Z494" s="2" t="inlineStr"/>
+      <c r="AA494" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/cecilia-becerra-becerra-0b7a2a29a</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="inlineStr">
+        <is>
+          <t>Entreviñas</t>
+        </is>
+      </c>
+      <c r="B495" s="2" t="inlineStr"/>
+      <c r="C495" s="2" t="inlineStr">
+        <is>
+          <t>168613</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E495" s="2" t="inlineStr">
+        <is>
+          <t>Zapopan</t>
+        </is>
+      </c>
+      <c r="F495" s="2" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G495" s="2" t="inlineStr">
+        <is>
+          <t>Calle Xicotencatl 153, Colonia Ciudad Del Sol</t>
+        </is>
+      </c>
+      <c r="H495" s="2" t="inlineStr">
+        <is>
+          <t>45050</t>
+        </is>
+      </c>
+      <c r="I495" s="2" t="inlineStr">
+        <is>
+          <t>https://www.entrevinas.store</t>
+        </is>
+      </c>
+      <c r="J495" s="2" t="inlineStr"/>
+      <c r="K495" s="2" t="inlineStr"/>
+      <c r="L495" s="2" t="inlineStr"/>
+      <c r="M495" s="2" t="inlineStr"/>
+      <c r="N495" s="2" t="inlineStr">
+        <is>
+          <t>entrevinas@gmail.com</t>
+        </is>
+      </c>
+      <c r="O495" s="2" t="inlineStr">
+        <is>
+          <t>+52 33 3121 5960</t>
+        </is>
+      </c>
+      <c r="P495" s="2" t="inlineStr"/>
+      <c r="Q495" s="2" t="inlineStr"/>
+      <c r="R495" s="2" t="inlineStr"/>
+      <c r="S495" s="2" t="inlineStr"/>
+      <c r="T495" s="2" t="inlineStr"/>
+      <c r="U495" s="2" t="inlineStr"/>
+      <c r="V495" s="2" t="inlineStr"/>
+      <c r="W495" s="2" t="inlineStr"/>
+      <c r="X495" s="2" t="inlineStr"/>
+      <c r="Y495" s="2" t="inlineStr"/>
+      <c r="Z495" s="2" t="inlineStr"/>
+      <c r="AA495" s="2" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>La Cava del Sumiller S.A. de C.V.</t>
+        </is>
+      </c>
+      <c r="B496" s="2" t="inlineStr"/>
+      <c r="C496" s="2" t="inlineStr">
+        <is>
+          <t>168612</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E496" s="2" t="inlineStr">
+        <is>
+          <t>Mérida</t>
+        </is>
+      </c>
+      <c r="F496" s="2" t="inlineStr">
+        <is>
+          <t>Yucatán</t>
+        </is>
+      </c>
+      <c r="G496" s="2" t="inlineStr">
+        <is>
+          <t>Calle 32, 458. Local 6-1A Col. La Florida</t>
+        </is>
+      </c>
+      <c r="H496" s="2" t="inlineStr">
+        <is>
+          <t>97138</t>
+        </is>
+      </c>
+      <c r="I496" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacavadelsumiller.com</t>
+        </is>
+      </c>
+      <c r="J496" s="2" t="inlineStr"/>
+      <c r="K496" s="2" t="inlineStr"/>
+      <c r="L496" s="2" t="inlineStr"/>
+      <c r="M496" s="2" t="inlineStr"/>
+      <c r="N496" s="2" t="inlineStr">
+        <is>
+          <t>hola@lacavadelsumiller.com</t>
+        </is>
+      </c>
+      <c r="O496" s="2" t="inlineStr">
+        <is>
+          <t>+52 999 666 2091</t>
+        </is>
+      </c>
+      <c r="P496" s="2" t="inlineStr"/>
+      <c r="Q496" s="2" t="inlineStr"/>
+      <c r="R496" s="2" t="inlineStr"/>
+      <c r="S496" s="2" t="inlineStr"/>
+      <c r="T496" s="2" t="inlineStr"/>
+      <c r="U496" s="2" t="inlineStr"/>
+      <c r="V496" s="2" t="inlineStr"/>
+      <c r="W496" s="2" t="inlineStr">
+        <is>
+          <t>Aitor Payo</t>
+        </is>
+      </c>
+      <c r="X496" s="2" t="inlineStr">
+        <is>
+          <t>Founding Sommelier</t>
+        </is>
+      </c>
+      <c r="Y496" s="2" t="inlineStr"/>
+      <c r="Z496" s="2" t="inlineStr"/>
+      <c r="AA496" s="2" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="inlineStr">
+        <is>
+          <t>La Cava del Sumiller S.A. de C.V.</t>
+        </is>
+      </c>
+      <c r="B497" s="2" t="inlineStr"/>
+      <c r="C497" s="2" t="inlineStr">
+        <is>
+          <t>168612</t>
+        </is>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E497" s="2" t="inlineStr">
+        <is>
+          <t>Mérida</t>
+        </is>
+      </c>
+      <c r="F497" s="2" t="inlineStr">
+        <is>
+          <t>Yucatán</t>
+        </is>
+      </c>
+      <c r="G497" s="2" t="inlineStr">
+        <is>
+          <t>Calle 32, 458. Local 6-1A Col. La Florida</t>
+        </is>
+      </c>
+      <c r="H497" s="2" t="inlineStr">
+        <is>
+          <t>97138</t>
+        </is>
+      </c>
+      <c r="I497" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacavadelsumiller.com</t>
+        </is>
+      </c>
+      <c r="J497" s="2" t="inlineStr"/>
+      <c r="K497" s="2" t="inlineStr"/>
+      <c r="L497" s="2" t="inlineStr"/>
+      <c r="M497" s="2" t="inlineStr"/>
+      <c r="N497" s="2" t="inlineStr">
+        <is>
+          <t>hola@lacavadelsumiller.com</t>
+        </is>
+      </c>
+      <c r="O497" s="2" t="inlineStr">
+        <is>
+          <t>+52 999 666 2091</t>
+        </is>
+      </c>
+      <c r="P497" s="2" t="inlineStr"/>
+      <c r="Q497" s="2" t="inlineStr"/>
+      <c r="R497" s="2" t="inlineStr"/>
+      <c r="S497" s="2" t="inlineStr"/>
+      <c r="T497" s="2" t="inlineStr"/>
+      <c r="U497" s="2" t="inlineStr"/>
+      <c r="V497" s="2" t="inlineStr"/>
+      <c r="W497" s="2" t="inlineStr">
+        <is>
+          <t>Lucia Fragoso</t>
+        </is>
+      </c>
+      <c r="X497" s="2" t="inlineStr">
+        <is>
+          <t>Sommelier</t>
+        </is>
+      </c>
+      <c r="Y497" s="2" t="inlineStr"/>
+      <c r="Z497" s="2" t="inlineStr"/>
+      <c r="AA497" s="2" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>La Cava del Sumiller S.A. de C.V.</t>
+        </is>
+      </c>
+      <c r="B498" s="2" t="inlineStr"/>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>168612</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>Mérida</t>
+        </is>
+      </c>
+      <c r="F498" s="2" t="inlineStr">
+        <is>
+          <t>Yucatán</t>
+        </is>
+      </c>
+      <c r="G498" s="2" t="inlineStr">
+        <is>
+          <t>Calle 32, 458. Local 6-1A Col. La Florida</t>
+        </is>
+      </c>
+      <c r="H498" s="2" t="inlineStr">
+        <is>
+          <t>97138</t>
+        </is>
+      </c>
+      <c r="I498" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacavadelsumiller.com</t>
+        </is>
+      </c>
+      <c r="J498" s="2" t="inlineStr"/>
+      <c r="K498" s="2" t="inlineStr"/>
+      <c r="L498" s="2" t="inlineStr"/>
+      <c r="M498" s="2" t="inlineStr"/>
+      <c r="N498" s="2" t="inlineStr">
+        <is>
+          <t>hola@lacavadelsumiller.com</t>
+        </is>
+      </c>
+      <c r="O498" s="2" t="inlineStr">
+        <is>
+          <t>+52 999 666 2091</t>
+        </is>
+      </c>
+      <c r="P498" s="2" t="inlineStr"/>
+      <c r="Q498" s="2" t="inlineStr"/>
+      <c r="R498" s="2" t="inlineStr"/>
+      <c r="S498" s="2" t="inlineStr"/>
+      <c r="T498" s="2" t="inlineStr"/>
+      <c r="U498" s="2" t="inlineStr"/>
+      <c r="V498" s="2" t="inlineStr"/>
+      <c r="W498" s="2" t="inlineStr">
+        <is>
+          <t>Valente García de Quevedo</t>
+        </is>
+      </c>
+      <c r="X498" s="2" t="inlineStr">
+        <is>
+          <t>Sommelier</t>
+        </is>
+      </c>
+      <c r="Y498" s="2" t="inlineStr"/>
+      <c r="Z498" s="2" t="inlineStr"/>
+      <c r="AA498" s="2" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="inlineStr">
+        <is>
+          <t>ABARROTERA DEL DUERO SA DE CV.</t>
+        </is>
+      </c>
+      <c r="B499" s="2" t="inlineStr">
+        <is>
+          <t>Duero Mayoreo</t>
+        </is>
+      </c>
+      <c r="C499" s="2" t="inlineStr">
+        <is>
+          <t>168611</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>Zamora</t>
+        </is>
+      </c>
+      <c r="F499" s="2" t="inlineStr">
+        <is>
+          <t>Michoacán</t>
+        </is>
+      </c>
+      <c r="G499" s="2" t="inlineStr">
+        <is>
+          <t>Av del Arbol #1200, Infonavit Arboledas</t>
+        </is>
+      </c>
+      <c r="H499" s="2" t="inlineStr"/>
+      <c r="I499" s="2" t="inlineStr">
+        <is>
+          <t>https://dueromayoreo.com</t>
+        </is>
+      </c>
+      <c r="J499" s="2" t="inlineStr"/>
+      <c r="K499" s="2" t="inlineStr"/>
+      <c r="L499" s="2" t="inlineStr"/>
+      <c r="M499" s="2" t="inlineStr"/>
+      <c r="N499" s="2" t="inlineStr">
+        <is>
+          <t>dueropremia@merza.com</t>
+        </is>
+      </c>
+      <c r="O499" s="2" t="inlineStr"/>
+      <c r="P499" s="2" t="inlineStr"/>
+      <c r="Q499" s="2" t="inlineStr"/>
+      <c r="R499" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/abarrotera-del-duero/</t>
+        </is>
+      </c>
+      <c r="S499" s="2" t="inlineStr"/>
+      <c r="T499" s="2" t="inlineStr"/>
+      <c r="U499" s="2" t="inlineStr"/>
+      <c r="V499" s="2" t="inlineStr"/>
+      <c r="W499" s="2" t="inlineStr">
+        <is>
+          <t>Paulina Chavez Martinez</t>
+        </is>
+      </c>
+      <c r="X499" s="2" t="inlineStr">
+        <is>
+          <t>Purchasing Analyst</t>
+        </is>
+      </c>
+      <c r="Y499" s="2" t="inlineStr"/>
+      <c r="Z499" s="2" t="inlineStr"/>
+      <c r="AA499" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/paulina-guadalupe-chavez-martinez-4016421a4</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>ABARROTERA DEL DUERO SA DE CV.</t>
+        </is>
+      </c>
+      <c r="B500" s="2" t="inlineStr">
+        <is>
+          <t>Duero Mayoreo</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>168611</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="inlineStr">
+        <is>
+          <t>Zamora</t>
+        </is>
+      </c>
+      <c r="F500" s="2" t="inlineStr">
+        <is>
+          <t>Michoacán</t>
+        </is>
+      </c>
+      <c r="G500" s="2" t="inlineStr">
+        <is>
+          <t>Av del Arbol #1200, Infonavit Arboledas</t>
+        </is>
+      </c>
+      <c r="H500" s="2" t="inlineStr"/>
+      <c r="I500" s="2" t="inlineStr">
+        <is>
+          <t>https://dueromayoreo.com</t>
+        </is>
+      </c>
+      <c r="J500" s="2" t="inlineStr"/>
+      <c r="K500" s="2" t="inlineStr"/>
+      <c r="L500" s="2" t="inlineStr"/>
+      <c r="M500" s="2" t="inlineStr"/>
+      <c r="N500" s="2" t="inlineStr">
+        <is>
+          <t>dueropremia@merza.com</t>
+        </is>
+      </c>
+      <c r="O500" s="2" t="inlineStr"/>
+      <c r="P500" s="2" t="inlineStr"/>
+      <c r="Q500" s="2" t="inlineStr"/>
+      <c r="R500" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/abarrotera-del-duero/</t>
+        </is>
+      </c>
+      <c r="S500" s="2" t="inlineStr"/>
+      <c r="T500" s="2" t="inlineStr"/>
+      <c r="U500" s="2" t="inlineStr"/>
+      <c r="V500" s="2" t="inlineStr"/>
+      <c r="W500" s="2" t="inlineStr">
+        <is>
+          <t>Luis Perez Magdaleno</t>
+        </is>
+      </c>
+      <c r="X500" s="2" t="inlineStr">
+        <is>
+          <t>Purchasing Manager</t>
+        </is>
+      </c>
+      <c r="Y500" s="2" t="inlineStr"/>
+      <c r="Z500" s="2" t="inlineStr"/>
+      <c r="AA500" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/luis-alejandro-p%c3%a9rez-magdaleno-b0b0051b2</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="inlineStr">
+        <is>
+          <t>ABARROTERA DEL DUERO SA DE CV.</t>
+        </is>
+      </c>
+      <c r="B501" s="2" t="inlineStr">
+        <is>
+          <t>Duero Mayoreo</t>
+        </is>
+      </c>
+      <c r="C501" s="2" t="inlineStr">
+        <is>
+          <t>168611</t>
+        </is>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E501" s="2" t="inlineStr">
+        <is>
+          <t>Zamora</t>
+        </is>
+      </c>
+      <c r="F501" s="2" t="inlineStr">
+        <is>
+          <t>Michoacán</t>
+        </is>
+      </c>
+      <c r="G501" s="2" t="inlineStr">
+        <is>
+          <t>Av del Arbol #1200, Infonavit Arboledas</t>
+        </is>
+      </c>
+      <c r="H501" s="2" t="inlineStr"/>
+      <c r="I501" s="2" t="inlineStr">
+        <is>
+          <t>https://dueromayoreo.com</t>
+        </is>
+      </c>
+      <c r="J501" s="2" t="inlineStr"/>
+      <c r="K501" s="2" t="inlineStr"/>
+      <c r="L501" s="2" t="inlineStr"/>
+      <c r="M501" s="2" t="inlineStr"/>
+      <c r="N501" s="2" t="inlineStr">
+        <is>
+          <t>dueropremia@merza.com</t>
+        </is>
+      </c>
+      <c r="O501" s="2" t="inlineStr"/>
+      <c r="P501" s="2" t="inlineStr"/>
+      <c r="Q501" s="2" t="inlineStr"/>
+      <c r="R501" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/abarrotera-del-duero/</t>
+        </is>
+      </c>
+      <c r="S501" s="2" t="inlineStr"/>
+      <c r="T501" s="2" t="inlineStr"/>
+      <c r="U501" s="2" t="inlineStr"/>
+      <c r="V501" s="2" t="inlineStr"/>
+      <c r="W501" s="2" t="inlineStr">
+        <is>
+          <t>Jose Viveros Lopez</t>
+        </is>
+      </c>
+      <c r="X501" s="2" t="inlineStr">
+        <is>
+          <t>Sales Consultant</t>
+        </is>
+      </c>
+      <c r="Y501" s="2" t="inlineStr"/>
+      <c r="Z501" s="2" t="inlineStr"/>
+      <c r="AA501" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/jose-antonio-viveros-lopez-a367a1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>ABARROTERA DEL DUERO SA DE CV.</t>
+        </is>
+      </c>
+      <c r="B502" s="2" t="inlineStr">
+        <is>
+          <t>Duero Mayoreo</t>
+        </is>
+      </c>
+      <c r="C502" s="2" t="inlineStr">
+        <is>
+          <t>168611</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E502" s="2" t="inlineStr">
+        <is>
+          <t>Zamora</t>
+        </is>
+      </c>
+      <c r="F502" s="2" t="inlineStr">
+        <is>
+          <t>Michoacán</t>
+        </is>
+      </c>
+      <c r="G502" s="2" t="inlineStr">
+        <is>
+          <t>Av del Arbol #1200, Infonavit Arboledas</t>
+        </is>
+      </c>
+      <c r="H502" s="2" t="inlineStr"/>
+      <c r="I502" s="2" t="inlineStr">
+        <is>
+          <t>https://dueromayoreo.com</t>
+        </is>
+      </c>
+      <c r="J502" s="2" t="inlineStr"/>
+      <c r="K502" s="2" t="inlineStr"/>
+      <c r="L502" s="2" t="inlineStr"/>
+      <c r="M502" s="2" t="inlineStr"/>
+      <c r="N502" s="2" t="inlineStr">
+        <is>
+          <t>dueropremia@merza.com</t>
+        </is>
+      </c>
+      <c r="O502" s="2" t="inlineStr"/>
+      <c r="P502" s="2" t="inlineStr"/>
+      <c r="Q502" s="2" t="inlineStr"/>
+      <c r="R502" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/abarrotera-del-duero/</t>
+        </is>
+      </c>
+      <c r="S502" s="2" t="inlineStr"/>
+      <c r="T502" s="2" t="inlineStr"/>
+      <c r="U502" s="2" t="inlineStr"/>
+      <c r="V502" s="2" t="inlineStr"/>
+      <c r="W502" s="2" t="inlineStr">
+        <is>
+          <t>Ricardo Gomez</t>
+        </is>
+      </c>
+      <c r="X502" s="2" t="inlineStr">
+        <is>
+          <t>Sales Supervisor</t>
+        </is>
+      </c>
+      <c r="Y502" s="2" t="inlineStr"/>
+      <c r="Z502" s="2" t="inlineStr"/>
+      <c r="AA502" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/ricardo-g%c3%b3mez-642913123</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="inlineStr">
+        <is>
+          <t>La Escocesa</t>
+        </is>
+      </c>
+      <c r="B503" s="2" t="inlineStr"/>
+      <c r="C503" s="2" t="inlineStr">
+        <is>
+          <t>168610</t>
+        </is>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E503" s="2" t="inlineStr">
+        <is>
+          <t>Cabo San Lucas</t>
+        </is>
+      </c>
+      <c r="F503" s="2" t="inlineStr">
+        <is>
+          <t>Baja California Sur</t>
+        </is>
+      </c>
+      <c r="G503" s="2" t="inlineStr">
+        <is>
+          <t>Muelle 20-34 / Puerta 2, 3 y 4, Frente a Breathless Hotel, Colonia El Medano</t>
+        </is>
+      </c>
+      <c r="H503" s="2" t="inlineStr">
+        <is>
+          <t>23450</t>
+        </is>
+      </c>
+      <c r="I503" s="2" t="inlineStr">
+        <is>
+          <t>https://laescocesa.com</t>
+        </is>
+      </c>
+      <c r="J503" s="2" t="inlineStr"/>
+      <c r="K503" s="2" t="inlineStr"/>
+      <c r="L503" s="2" t="inlineStr"/>
+      <c r="M503" s="2" t="inlineStr"/>
+      <c r="N503" s="2" t="inlineStr"/>
+      <c r="O503" s="2" t="inlineStr"/>
+      <c r="P503" s="2" t="inlineStr"/>
+      <c r="Q503" s="2" t="inlineStr"/>
+      <c r="R503" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/la-escocesa-mx</t>
+        </is>
+      </c>
+      <c r="S503" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/LaEscocesaVinos</t>
+        </is>
+      </c>
+      <c r="T503" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/laescocesavinos/</t>
+        </is>
+      </c>
+      <c r="U503" s="2" t="inlineStr"/>
+      <c r="V503" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@LaEscocesaVinos</t>
+        </is>
+      </c>
+      <c r="W503" s="2" t="inlineStr">
+        <is>
+          <t>César Julián Osuna Martínez</t>
+        </is>
+      </c>
+      <c r="X503" s="2" t="inlineStr">
+        <is>
+          <t>Ceo</t>
+        </is>
+      </c>
+      <c r="Y503" s="2" t="inlineStr"/>
+      <c r="Z503" s="2" t="inlineStr"/>
+      <c r="AA503" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/c%C3%A9sar-juli%C3%A1n-osuna-mart%C3%ADnez-45985862/</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>La Escocesa</t>
+        </is>
+      </c>
+      <c r="B504" s="2" t="inlineStr"/>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>168610</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E504" s="2" t="inlineStr">
+        <is>
+          <t>Cabo San Lucas</t>
+        </is>
+      </c>
+      <c r="F504" s="2" t="inlineStr">
+        <is>
+          <t>Baja California Sur</t>
+        </is>
+      </c>
+      <c r="G504" s="2" t="inlineStr">
+        <is>
+          <t>Muelle 20-34 / Puerta 2, 3 y 4, Frente a Breathless Hotel, Colonia El Medano</t>
+        </is>
+      </c>
+      <c r="H504" s="2" t="inlineStr">
+        <is>
+          <t>23450</t>
+        </is>
+      </c>
+      <c r="I504" s="2" t="inlineStr">
+        <is>
+          <t>https://laescocesa.com</t>
+        </is>
+      </c>
+      <c r="J504" s="2" t="inlineStr"/>
+      <c r="K504" s="2" t="inlineStr"/>
+      <c r="L504" s="2" t="inlineStr"/>
+      <c r="M504" s="2" t="inlineStr"/>
+      <c r="N504" s="2" t="inlineStr"/>
+      <c r="O504" s="2" t="inlineStr"/>
+      <c r="P504" s="2" t="inlineStr"/>
+      <c r="Q504" s="2" t="inlineStr"/>
+      <c r="R504" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/la-escocesa-mx</t>
+        </is>
+      </c>
+      <c r="S504" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/LaEscocesaVinos</t>
+        </is>
+      </c>
+      <c r="T504" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/laescocesavinos/</t>
+        </is>
+      </c>
+      <c r="U504" s="2" t="inlineStr"/>
+      <c r="V504" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@LaEscocesaVinos</t>
+        </is>
+      </c>
+      <c r="W504" s="2" t="inlineStr">
+        <is>
+          <t>Vianey Gaytan</t>
+        </is>
+      </c>
+      <c r="X504" s="2" t="inlineStr">
+        <is>
+          <t>Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="Y504" s="2" t="inlineStr"/>
+      <c r="Z504" s="2" t="inlineStr"/>
+      <c r="AA504" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/vianey-gaytan-a613ba189</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="inlineStr">
+        <is>
+          <t>Vinolandia</t>
+        </is>
+      </c>
+      <c r="B505" s="2" t="inlineStr"/>
+      <c r="C505" s="2" t="inlineStr">
+        <is>
+          <t>168609</t>
+        </is>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E505" s="2" t="inlineStr">
+        <is>
+          <t>Orizaba</t>
+        </is>
+      </c>
+      <c r="F505" s="2" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+      <c r="G505" s="2" t="inlineStr">
+        <is>
+          <t>Poniente 6 Núm. 82 Centro</t>
+        </is>
+      </c>
+      <c r="H505" s="2" t="inlineStr">
+        <is>
+          <t>94300</t>
+        </is>
+      </c>
+      <c r="I505" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vinolandia.com.mx</t>
+        </is>
+      </c>
+      <c r="J505" s="2" t="inlineStr"/>
+      <c r="K505" s="2" t="inlineStr"/>
+      <c r="L505" s="2" t="inlineStr"/>
+      <c r="M505" s="2" t="inlineStr"/>
+      <c r="N505" s="2" t="inlineStr">
+        <is>
+          <t>vinolandia_orizaba@hotmail.com</t>
+        </is>
+      </c>
+      <c r="O505" s="2" t="inlineStr">
+        <is>
+          <t>+52 272 725 0707</t>
+        </is>
+      </c>
+      <c r="P505" s="2" t="inlineStr"/>
+      <c r="Q505" s="2" t="inlineStr"/>
+      <c r="R505" s="2" t="inlineStr"/>
+      <c r="S505" s="2" t="inlineStr">
+        <is>
+          <t>https://facebook.com/vinolandiaorizabaoficial/?locale=es_LA</t>
+        </is>
+      </c>
+      <c r="T505" s="2" t="inlineStr">
+        <is>
+          <t>https://instagram.com/vinolandiaorizaba</t>
+        </is>
+      </c>
+      <c r="U505" s="2" t="inlineStr"/>
+      <c r="V505" s="2" t="inlineStr"/>
+      <c r="W505" s="2" t="inlineStr"/>
+      <c r="X505" s="2" t="inlineStr"/>
+      <c r="Y505" s="2" t="inlineStr"/>
+      <c r="Z505" s="2" t="inlineStr"/>
+      <c r="AA505" s="2" t="inlineStr"/>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>Grupo El Valor</t>
+        </is>
+      </c>
+      <c r="B506" s="2" t="inlineStr"/>
+      <c r="C506" s="2" t="inlineStr">
+        <is>
+          <t>168608</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E506" s="2" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="F506" s="2" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G506" s="2" t="inlineStr">
+        <is>
+          <t>Av. Del Mercado #1566 Mercado de Abastos</t>
+        </is>
+      </c>
+      <c r="H506" s="2" t="inlineStr"/>
+      <c r="I506" s="2" t="inlineStr">
+        <is>
+          <t>https://elvalor.mx</t>
+        </is>
+      </c>
+      <c r="J506" s="2" t="inlineStr"/>
+      <c r="K506" s="2" t="inlineStr"/>
+      <c r="L506" s="2" t="inlineStr"/>
+      <c r="M506" s="2" t="inlineStr"/>
+      <c r="N506" s="2" t="inlineStr">
+        <is>
+          <t>ventaenlinea@grupoelvalor.com</t>
+        </is>
+      </c>
+      <c r="O506" s="2" t="inlineStr"/>
+      <c r="P506" s="2" t="inlineStr"/>
+      <c r="Q506" s="2" t="inlineStr"/>
+      <c r="R506" s="2" t="inlineStr"/>
+      <c r="S506" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/bodegaselvalor</t>
+        </is>
+      </c>
+      <c r="T506" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elvalor.comercializadora</t>
+        </is>
+      </c>
+      <c r="U506" s="2" t="inlineStr"/>
+      <c r="V506" s="2" t="inlineStr"/>
+      <c r="W506" s="2" t="inlineStr"/>
+      <c r="X506" s="2" t="inlineStr"/>
+      <c r="Y506" s="2" t="inlineStr"/>
+      <c r="Z506" s="2" t="inlineStr"/>
+      <c r="AA506" s="2" t="inlineStr"/>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cava Grapaan </t>
+        </is>
+      </c>
+      <c r="B507" s="2" t="inlineStr"/>
+      <c r="C507" s="2" t="inlineStr">
+        <is>
+          <t>168607</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>Boca del Río</t>
+        </is>
+      </c>
+      <c r="F507" s="2" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+      <c r="G507" s="2" t="inlineStr">
+        <is>
+          <t>Bv. Adolfo Ruíz Cortines</t>
+        </is>
+      </c>
+      <c r="H507" s="2" t="inlineStr">
+        <is>
+          <t>94299</t>
+        </is>
+      </c>
+      <c r="I507" s="2" t="inlineStr">
+        <is>
+          <t>https://cavagrapaan.alvisar.com</t>
+        </is>
+      </c>
+      <c r="J507" s="2" t="inlineStr"/>
+      <c r="K507" s="2" t="inlineStr"/>
+      <c r="L507" s="2" t="inlineStr"/>
+      <c r="M507" s="2" t="inlineStr"/>
+      <c r="N507" s="2" t="inlineStr">
+        <is>
+          <t>ventas@alvisar.com</t>
+        </is>
+      </c>
+      <c r="O507" s="2" t="inlineStr">
+        <is>
+          <t>+52 232 324 9900</t>
+        </is>
+      </c>
+      <c r="P507" s="2" t="inlineStr"/>
+      <c r="Q507" s="2" t="inlineStr"/>
+      <c r="R507" s="2" t="inlineStr"/>
+      <c r="S507" s="2" t="inlineStr"/>
+      <c r="T507" s="2" t="inlineStr"/>
+      <c r="U507" s="2" t="inlineStr"/>
+      <c r="V507" s="2" t="inlineStr"/>
+      <c r="W507" s="2" t="inlineStr"/>
+      <c r="X507" s="2" t="inlineStr"/>
+      <c r="Y507" s="2" t="inlineStr"/>
+      <c r="Z507" s="2" t="inlineStr"/>
+      <c r="AA507" s="2" t="inlineStr"/>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>VIMART</t>
+        </is>
+      </c>
+      <c r="B508" s="2" t="inlineStr"/>
+      <c r="C508" s="2" t="inlineStr">
+        <is>
+          <t>168606</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E508" s="2" t="inlineStr">
+        <is>
+          <t>Oaxaca de Juárez</t>
+        </is>
+      </c>
+      <c r="F508" s="2" t="inlineStr">
+        <is>
+          <t>Oaxaca</t>
+        </is>
+      </c>
+      <c r="G508" s="2" t="inlineStr">
+        <is>
+          <t>Avenida Las Etnias 103 B Colonia Olímpica</t>
+        </is>
+      </c>
+      <c r="H508" s="2" t="inlineStr">
+        <is>
+          <t>68044</t>
+        </is>
+      </c>
+      <c r="I508" s="2" t="inlineStr">
+        <is>
+          <t>https://vimart.mx</t>
+        </is>
+      </c>
+      <c r="J508" s="2" t="inlineStr"/>
+      <c r="K508" s="2" t="inlineStr"/>
+      <c r="L508" s="2" t="inlineStr"/>
+      <c r="M508" s="2" t="inlineStr"/>
+      <c r="N508" s="2" t="inlineStr">
+        <is>
+          <t>vimart.pedidos@gmail.com</t>
+        </is>
+      </c>
+      <c r="O508" s="2" t="inlineStr">
+        <is>
+          <t>+52 951 516 9810</t>
+        </is>
+      </c>
+      <c r="P508" s="2" t="inlineStr"/>
+      <c r="Q508" s="2" t="inlineStr"/>
+      <c r="R508" s="2" t="inlineStr"/>
+      <c r="S508" s="2" t="inlineStr"/>
+      <c r="T508" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vimartmx/</t>
+        </is>
+      </c>
+      <c r="U508" s="2" t="inlineStr"/>
+      <c r="V508" s="2" t="inlineStr"/>
+      <c r="W508" s="2" t="inlineStr"/>
+      <c r="X508" s="2" t="inlineStr"/>
+      <c r="Y508" s="2" t="inlineStr"/>
+      <c r="Z508" s="2" t="inlineStr"/>
+      <c r="AA508" s="2" t="inlineStr"/>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>Manjar's S.A. de C.V.</t>
+        </is>
+      </c>
+      <c r="B509" s="2" t="inlineStr"/>
+      <c r="C509" s="2" t="inlineStr">
+        <is>
+          <t>168605</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E509" s="2" t="inlineStr">
+        <is>
+          <t>Boca del Río</t>
+        </is>
+      </c>
+      <c r="F509" s="2" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+      <c r="G509" s="2" t="inlineStr">
+        <is>
+          <t>Blvd. del Mar 368</t>
+        </is>
+      </c>
+      <c r="H509" s="2" t="inlineStr"/>
+      <c r="I509" s="2" t="inlineStr">
+        <is>
+          <t>https://manjars.com</t>
+        </is>
+      </c>
+      <c r="J509" s="2" t="inlineStr"/>
+      <c r="K509" s="2" t="inlineStr"/>
+      <c r="L509" s="2" t="inlineStr"/>
+      <c r="M509" s="2" t="inlineStr"/>
+      <c r="N509" s="2" t="inlineStr">
+        <is>
+          <t>manjarsveracruz@gmail.com</t>
+        </is>
+      </c>
+      <c r="O509" s="2" t="inlineStr">
+        <is>
+          <t>+52 229 921 8011</t>
+        </is>
+      </c>
+      <c r="P509" s="2" t="inlineStr"/>
+      <c r="Q509" s="2" t="inlineStr"/>
+      <c r="R509" s="2" t="inlineStr"/>
+      <c r="S509" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/manjarsveracruz</t>
+        </is>
+      </c>
+      <c r="T509" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/manjars_ver</t>
+        </is>
+      </c>
+      <c r="U509" s="2" t="inlineStr"/>
+      <c r="V509" s="2" t="inlineStr"/>
+      <c r="W509" s="2" t="inlineStr"/>
+      <c r="X509" s="2" t="inlineStr"/>
+      <c r="Y509" s="2" t="inlineStr"/>
+      <c r="Z509" s="2" t="inlineStr"/>
+      <c r="AA509" s="2" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>Teravino</t>
+        </is>
+      </c>
+      <c r="B510" s="2" t="inlineStr"/>
+      <c r="C510" s="2" t="inlineStr">
+        <is>
+          <t>168604</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E510" s="2" t="inlineStr">
+        <is>
+          <t>San José del Cabo</t>
+        </is>
+      </c>
+      <c r="F510" s="2" t="inlineStr">
+        <is>
+          <t>Baja California Sur</t>
+        </is>
+      </c>
+      <c r="G510" s="2" t="inlineStr">
+        <is>
+          <t>Carr. Transp. Km 43.5</t>
+        </is>
+      </c>
+      <c r="H510" s="2" t="inlineStr">
+        <is>
+          <t>23400</t>
+        </is>
+      </c>
+      <c r="I510" s="2" t="inlineStr">
+        <is>
+          <t>https://www.teravino.com</t>
+        </is>
+      </c>
+      <c r="J510" s="2" t="inlineStr"/>
+      <c r="K510" s="2" t="inlineStr"/>
+      <c r="L510" s="2" t="inlineStr"/>
+      <c r="M510" s="2" t="inlineStr"/>
+      <c r="N510" s="2" t="inlineStr">
+        <is>
+          <t>sabrina@teravino.com</t>
+        </is>
+      </c>
+      <c r="O510" s="2" t="inlineStr">
+        <is>
+          <t>+52 624 172 3702</t>
+        </is>
+      </c>
+      <c r="P510" s="2" t="inlineStr"/>
+      <c r="Q510" s="2" t="inlineStr"/>
+      <c r="R510" s="2" t="inlineStr"/>
+      <c r="S510" s="2" t="inlineStr"/>
+      <c r="T510" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/teravinowine/</t>
+        </is>
+      </c>
+      <c r="U510" s="2" t="inlineStr"/>
+      <c r="V510" s="2" t="inlineStr"/>
+      <c r="W510" s="2" t="inlineStr">
+        <is>
+          <t>Sabrina A Sanchez G</t>
+        </is>
+      </c>
+      <c r="X510" s="2" t="inlineStr">
+        <is>
+          <t>Ceo</t>
+        </is>
+      </c>
+      <c r="Y510" s="2" t="inlineStr"/>
+      <c r="Z510" s="2" t="inlineStr"/>
+      <c r="AA510" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sabrina-a-sanchez-g-73a14335</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="inlineStr">
+        <is>
+          <t>Salvaje Vinos (BC Selections)</t>
+        </is>
+      </c>
+      <c r="B511" s="2" t="inlineStr"/>
+      <c r="C511" s="2" t="inlineStr">
+        <is>
+          <t>168600</t>
+        </is>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E511" s="2" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+      <c r="F511" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo Leon</t>
+        </is>
+      </c>
+      <c r="G511" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Bernardo Nobel 2108 Col. Country Sol</t>
+        </is>
+      </c>
+      <c r="H511" s="2" t="inlineStr">
+        <is>
+          <t>67174</t>
+        </is>
+      </c>
+      <c r="I511" s="2" t="inlineStr">
+        <is>
+          <t>https://www.salvajevinos.com</t>
+        </is>
+      </c>
+      <c r="J511" s="2" t="inlineStr"/>
+      <c r="K511" s="2" t="inlineStr"/>
+      <c r="L511" s="2" t="inlineStr"/>
+      <c r="M511" s="2" t="inlineStr"/>
+      <c r="N511" s="2" t="inlineStr">
+        <is>
+          <t>hola@salvajevinos.com</t>
+        </is>
+      </c>
+      <c r="O511" s="2" t="inlineStr"/>
+      <c r="P511" s="2" t="inlineStr"/>
+      <c r="Q511" s="2" t="inlineStr"/>
+      <c r="R511" s="2" t="inlineStr"/>
+      <c r="S511" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SalvajeVinosMx</t>
+        </is>
+      </c>
+      <c r="T511" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/salvajevinos</t>
+        </is>
+      </c>
+      <c r="U511" s="2" t="inlineStr"/>
+      <c r="V511" s="2" t="inlineStr"/>
+      <c r="W511" s="2" t="inlineStr"/>
+      <c r="X511" s="2" t="inlineStr"/>
+      <c r="Y511" s="2" t="inlineStr"/>
+      <c r="Z511" s="2" t="inlineStr"/>
+      <c r="AA511" s="2" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>ORFE</t>
+        </is>
+      </c>
+      <c r="B512" s="2" t="inlineStr"/>
+      <c r="C512" s="2" t="inlineStr">
+        <is>
+          <t>168599</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E512" s="2" t="inlineStr">
+        <is>
+          <t>Mexico City</t>
+        </is>
+      </c>
+      <c r="F512" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="G512" s="2" t="inlineStr">
+        <is>
+          <t>Campos Elíseos 176, piso 1, Polanco V Sección</t>
+        </is>
+      </c>
+      <c r="H512" s="2" t="inlineStr"/>
+      <c r="I512" s="2" t="inlineStr">
+        <is>
+          <t>https://orfemexico.com.mx</t>
+        </is>
+      </c>
+      <c r="J512" s="2" t="inlineStr"/>
+      <c r="K512" s="2" t="inlineStr"/>
+      <c r="L512" s="2" t="inlineStr"/>
+      <c r="M512" s="2" t="inlineStr"/>
+      <c r="N512" s="2" t="inlineStr">
+        <is>
+          <t>info@orfemexico.com.mx</t>
+        </is>
+      </c>
+      <c r="O512" s="2" t="inlineStr">
+        <is>
+          <t>+52 55 5543 9968</t>
+        </is>
+      </c>
+      <c r="P512" s="2" t="inlineStr"/>
+      <c r="Q512" s="2" t="inlineStr"/>
+      <c r="R512" s="2" t="inlineStr"/>
+      <c r="S512" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/OrfeMexico/</t>
+        </is>
+      </c>
+      <c r="T512" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/orfemexico/</t>
+        </is>
+      </c>
+      <c r="U512" s="2" t="inlineStr"/>
+      <c r="V512" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@orfemexico8941</t>
+        </is>
+      </c>
+      <c r="W512" s="2" t="inlineStr">
+        <is>
+          <t>Giovanni Orlotti</t>
+        </is>
+      </c>
+      <c r="X512" s="2" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="Y512" s="2" t="inlineStr"/>
+      <c r="Z512" s="2" t="inlineStr"/>
+      <c r="AA512" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/giovanni-orlotti-a361a137/</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="inlineStr">
+        <is>
+          <t>ORFE</t>
+        </is>
+      </c>
+      <c r="B513" s="2" t="inlineStr"/>
+      <c r="C513" s="2" t="inlineStr">
+        <is>
+          <t>168599</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E513" s="2" t="inlineStr">
+        <is>
+          <t>Mexico City</t>
+        </is>
+      </c>
+      <c r="F513" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="G513" s="2" t="inlineStr">
+        <is>
+          <t>Campos Elíseos 176, piso 1, Polanco V Sección</t>
+        </is>
+      </c>
+      <c r="H513" s="2" t="inlineStr"/>
+      <c r="I513" s="2" t="inlineStr">
+        <is>
+          <t>https://orfemexico.com.mx</t>
+        </is>
+      </c>
+      <c r="J513" s="2" t="inlineStr"/>
+      <c r="K513" s="2" t="inlineStr"/>
+      <c r="L513" s="2" t="inlineStr"/>
+      <c r="M513" s="2" t="inlineStr"/>
+      <c r="N513" s="2" t="inlineStr">
+        <is>
+          <t>info@orfemexico.com.mx</t>
+        </is>
+      </c>
+      <c r="O513" s="2" t="inlineStr">
+        <is>
+          <t>+52 55 5543 9968</t>
+        </is>
+      </c>
+      <c r="P513" s="2" t="inlineStr"/>
+      <c r="Q513" s="2" t="inlineStr"/>
+      <c r="R513" s="2" t="inlineStr"/>
+      <c r="S513" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/OrfeMexico/</t>
+        </is>
+      </c>
+      <c r="T513" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/orfemexico/</t>
+        </is>
+      </c>
+      <c r="U513" s="2" t="inlineStr"/>
+      <c r="V513" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@orfemexico8941</t>
+        </is>
+      </c>
+      <c r="W513" s="2" t="inlineStr">
+        <is>
+          <t>Francisco Olvera Islas</t>
+        </is>
+      </c>
+      <c r="X513" s="2" t="inlineStr">
+        <is>
+          <t>Logistics Manager</t>
+        </is>
+      </c>
+      <c r="Y513" s="2" t="inlineStr"/>
+      <c r="Z513" s="2" t="inlineStr"/>
+      <c r="AA513" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/francisco-olvera-islas-b023751b6</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>Grupo Vinimart</t>
+        </is>
+      </c>
+      <c r="B514" s="2" t="inlineStr"/>
+      <c r="C514" s="2" t="inlineStr">
+        <is>
+          <t>168598</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E514" s="2" t="inlineStr">
+        <is>
+          <t>Álvaro Obregón</t>
+        </is>
+      </c>
+      <c r="F514" s="2" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="G514" s="2" t="inlineStr">
+        <is>
+          <t>Av. Centenario 358-L1, Merced Gómez</t>
+        </is>
+      </c>
+      <c r="H514" s="2" t="inlineStr">
+        <is>
+          <t>01600</t>
+        </is>
+      </c>
+      <c r="I514" s="2" t="inlineStr">
+        <is>
+          <t>https://promowine.mx, https://vinimart.com.mx</t>
+        </is>
+      </c>
+      <c r="J514" s="2" t="inlineStr"/>
+      <c r="K514" s="2" t="inlineStr"/>
+      <c r="L514" s="2" t="inlineStr"/>
+      <c r="M514" s="2" t="inlineStr"/>
+      <c r="N514" s="2" t="inlineStr">
+        <is>
+          <t>rohu@vinimart.com.mx</t>
+        </is>
+      </c>
+      <c r="O514" s="2" t="inlineStr">
+        <is>
+          <t>+52 33 3110 0174</t>
+        </is>
+      </c>
+      <c r="P514" s="2" t="inlineStr"/>
+      <c r="Q514" s="2" t="inlineStr"/>
+      <c r="R514" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupovinimart/</t>
+        </is>
+      </c>
+      <c r="S514" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/PROMOWINE/</t>
+        </is>
+      </c>
+      <c r="T514" s="2" t="inlineStr">
+        <is>
+          <t>https://instagram.com/grupovinimart</t>
+        </is>
+      </c>
+      <c r="U514" s="2" t="inlineStr"/>
+      <c r="V514" s="2" t="inlineStr"/>
+      <c r="W514" s="2" t="inlineStr">
+        <is>
+          <t>Rodrigo Rodriguez Huerta</t>
+        </is>
+      </c>
+      <c r="X514" s="2" t="inlineStr">
+        <is>
+          <t>Import and Product Manager</t>
+        </is>
+      </c>
+      <c r="Y514" s="2" t="inlineStr"/>
+      <c r="Z514" s="2" t="inlineStr"/>
+      <c r="AA514" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rodrigo-rodriguez-huerta-9710b7126/</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>Vinosapiens</t>
+        </is>
+      </c>
+      <c r="B515" s="2" t="inlineStr"/>
+      <c r="C515" s="2" t="inlineStr">
+        <is>
+          <t>168597</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E515" s="2" t="inlineStr">
+        <is>
+          <t>San Pedro Garza García</t>
+        </is>
+      </c>
+      <c r="F515" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G515" s="2" t="inlineStr">
+        <is>
+          <t>Calz. del Valle 409, Col. Del Valle</t>
+        </is>
+      </c>
+      <c r="H515" s="2" t="inlineStr">
+        <is>
+          <t>66220</t>
+        </is>
+      </c>
+      <c r="I515" s="2" t="inlineStr">
+        <is>
+          <t>https://vinosapiens.com</t>
+        </is>
+      </c>
+      <c r="J515" s="2" t="inlineStr"/>
+      <c r="K515" s="2" t="inlineStr"/>
+      <c r="L515" s="2" t="inlineStr"/>
+      <c r="M515" s="2" t="inlineStr"/>
+      <c r="N515" s="2" t="inlineStr">
+        <is>
+          <t>ventas@vinosapiens.com</t>
+        </is>
+      </c>
+      <c r="O515" s="2" t="inlineStr">
+        <is>
+          <t>+52 81 2315 2299</t>
+        </is>
+      </c>
+      <c r="P515" s="2" t="inlineStr"/>
+      <c r="Q515" s="2" t="inlineStr"/>
+      <c r="R515" s="2" t="inlineStr"/>
+      <c r="S515" s="2" t="inlineStr"/>
+      <c r="T515" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vinosapiens/</t>
+        </is>
+      </c>
+      <c r="U515" s="2" t="inlineStr"/>
+      <c r="V515" s="2" t="inlineStr"/>
+      <c r="W515" s="2" t="inlineStr"/>
+      <c r="X515" s="2" t="inlineStr"/>
+      <c r="Y515" s="2" t="inlineStr"/>
+      <c r="Z515" s="2" t="inlineStr"/>
+      <c r="AA515" s="2" t="inlineStr"/>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>Vino ConSentido</t>
+        </is>
+      </c>
+      <c r="B516" s="2" t="inlineStr"/>
+      <c r="C516" s="2" t="inlineStr">
+        <is>
+          <t>168596</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="F516" s="2" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="G516" s="2" t="inlineStr">
+        <is>
+          <t>Vértiz 847</t>
+        </is>
+      </c>
+      <c r="H516" s="2" t="inlineStr">
+        <is>
+          <t>03023</t>
+        </is>
+      </c>
+      <c r="I516" s="2" t="inlineStr">
+        <is>
+          <t>https://vinoconsentido.mx</t>
+        </is>
+      </c>
+      <c r="J516" s="2" t="inlineStr"/>
+      <c r="K516" s="2" t="inlineStr"/>
+      <c r="L516" s="2" t="inlineStr"/>
+      <c r="M516" s="2" t="inlineStr"/>
+      <c r="N516" s="2" t="inlineStr">
+        <is>
+          <t>contacto@vinoconsentido.mx</t>
+        </is>
+      </c>
+      <c r="O516" s="2" t="inlineStr"/>
+      <c r="P516" s="2" t="inlineStr"/>
+      <c r="Q516" s="2" t="inlineStr"/>
+      <c r="R516" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/viavinomx/</t>
+        </is>
+      </c>
+      <c r="S516" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/vinoconsentido.mx</t>
+        </is>
+      </c>
+      <c r="T516" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vinoconsentido.mx/</t>
+        </is>
+      </c>
+      <c r="U516" s="2" t="inlineStr"/>
+      <c r="V516" s="2" t="inlineStr"/>
+      <c r="W516" s="2" t="inlineStr">
+        <is>
+          <t>Erika Villanueva</t>
+        </is>
+      </c>
+      <c r="X516" s="2" t="inlineStr">
+        <is>
+          <t>Founding partner</t>
+        </is>
+      </c>
+      <c r="Y516" s="2" t="inlineStr"/>
+      <c r="Z516" s="2" t="inlineStr"/>
+      <c r="AA516" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/erika-esther-villanueva/</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>Vivo El Vino</t>
+        </is>
+      </c>
+      <c r="B517" s="2" t="inlineStr"/>
+      <c r="C517" s="2" t="inlineStr">
+        <is>
+          <t>168595</t>
+        </is>
+      </c>
+      <c r="D517" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E517" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Hidalgo</t>
+        </is>
+      </c>
+      <c r="F517" s="2" t="inlineStr">
+        <is>
+          <t>Ciudad de Mexico</t>
+        </is>
+      </c>
+      <c r="G517" s="2" t="inlineStr">
+        <is>
+          <t>Paseo de las Palmas 751 - 5 Col. Lomas de Chapultepec</t>
+        </is>
+      </c>
+      <c r="H517" s="2" t="inlineStr">
+        <is>
+          <t>11000</t>
+        </is>
+      </c>
+      <c r="I517" s="2" t="inlineStr">
+        <is>
+          <t>https://vivoelvino.com</t>
+        </is>
+      </c>
+      <c r="J517" s="2" t="inlineStr"/>
+      <c r="K517" s="2" t="inlineStr"/>
+      <c r="L517" s="2" t="inlineStr"/>
+      <c r="M517" s="2" t="inlineStr"/>
+      <c r="N517" s="2" t="inlineStr">
+        <is>
+          <t>comercial@vivoelvino.com.mx</t>
+        </is>
+      </c>
+      <c r="O517" s="2" t="inlineStr"/>
+      <c r="P517" s="2" t="inlineStr"/>
+      <c r="Q517" s="2" t="inlineStr"/>
+      <c r="R517" s="2" t="inlineStr"/>
+      <c r="S517" s="2" t="inlineStr"/>
+      <c r="T517" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vivoelvino.com.mx/</t>
+        </is>
+      </c>
+      <c r="U517" s="2" t="inlineStr"/>
+      <c r="V517" s="2" t="inlineStr"/>
+      <c r="W517" s="2" t="inlineStr"/>
+      <c r="X517" s="2" t="inlineStr"/>
+      <c r="Y517" s="2" t="inlineStr"/>
+      <c r="Z517" s="2" t="inlineStr"/>
+      <c r="AA517" s="2" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>Quercus Soluciones Comerciales</t>
+        </is>
+      </c>
+      <c r="B518" s="2" t="inlineStr"/>
+      <c r="C518" s="2" t="inlineStr">
+        <is>
+          <t>168594</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E518" s="2" t="inlineStr">
+        <is>
+          <t>Tizayuca</t>
+        </is>
+      </c>
+      <c r="F518" s="2" t="inlineStr">
+        <is>
+          <t>Hidalgo</t>
+        </is>
+      </c>
+      <c r="G518" s="2" t="inlineStr">
+        <is>
+          <t>Oriente 5 L21Mz7</t>
+        </is>
+      </c>
+      <c r="H518" s="2" t="inlineStr">
+        <is>
+          <t>43800</t>
+        </is>
+      </c>
+      <c r="I518" s="2" t="inlineStr">
+        <is>
+          <t>https://www.quercussoluciones.com, https://www.vinosdeeslovenia.com</t>
+        </is>
+      </c>
+      <c r="J518" s="2" t="inlineStr"/>
+      <c r="K518" s="2" t="inlineStr"/>
+      <c r="L518" s="2" t="inlineStr"/>
+      <c r="M518" s="2" t="inlineStr"/>
+      <c r="N518" s="2" t="inlineStr">
+        <is>
+          <t>administracion@quercussoluciones.com</t>
+        </is>
+      </c>
+      <c r="O518" s="2" t="inlineStr"/>
+      <c r="P518" s="2" t="inlineStr"/>
+      <c r="Q518" s="2" t="inlineStr"/>
+      <c r="R518" s="2" t="inlineStr"/>
+      <c r="S518" s="2" t="inlineStr"/>
+      <c r="T518" s="2" t="inlineStr"/>
+      <c r="U518" s="2" t="inlineStr"/>
+      <c r="V518" s="2" t="inlineStr"/>
+      <c r="W518" s="2" t="inlineStr"/>
+      <c r="X518" s="2" t="inlineStr"/>
+      <c r="Y518" s="2" t="inlineStr"/>
+      <c r="Z518" s="2" t="inlineStr"/>
+      <c r="AA518" s="2" t="inlineStr"/>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>Vino Para Todos</t>
+        </is>
+      </c>
+      <c r="B519" s="2" t="inlineStr"/>
+      <c r="C519" s="2" t="inlineStr">
+        <is>
+          <t>168593</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E519" s="2" t="inlineStr">
+        <is>
+          <t>Colima</t>
+        </is>
+      </c>
+      <c r="F519" s="2" t="inlineStr">
+        <is>
+          <t>Colima</t>
+        </is>
+      </c>
+      <c r="G519" s="2" t="inlineStr">
+        <is>
+          <t>Emilio Rabasa #327, Colonia Real Vista Hermosa III</t>
+        </is>
+      </c>
+      <c r="H519" s="2" t="inlineStr">
+        <is>
+          <t>28018</t>
+        </is>
+      </c>
+      <c r="I519" s="2" t="inlineStr">
+        <is>
+          <t>https://vinoparatodos.mx</t>
+        </is>
+      </c>
+      <c r="J519" s="2" t="inlineStr"/>
+      <c r="K519" s="2" t="inlineStr"/>
+      <c r="L519" s="2" t="inlineStr"/>
+      <c r="M519" s="2" t="inlineStr"/>
+      <c r="N519" s="2" t="inlineStr">
+        <is>
+          <t>atencionvpt@gmail.com</t>
+        </is>
+      </c>
+      <c r="O519" s="2" t="inlineStr"/>
+      <c r="P519" s="2" t="inlineStr"/>
+      <c r="Q519" s="2" t="inlineStr"/>
+      <c r="R519" s="2" t="inlineStr"/>
+      <c r="S519" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/vinoparatodosmx</t>
+        </is>
+      </c>
+      <c r="T519" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vinoparatodosmex/</t>
+        </is>
+      </c>
+      <c r="U519" s="2" t="inlineStr"/>
+      <c r="V519" s="2" t="inlineStr"/>
+      <c r="W519" s="2" t="inlineStr"/>
+      <c r="X519" s="2" t="inlineStr"/>
+      <c r="Y519" s="2" t="inlineStr"/>
+      <c r="Z519" s="2" t="inlineStr"/>
+      <c r="AA519" s="2" t="inlineStr"/>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>Basal Mayoreo</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="inlineStr"/>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>168592</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="F520" s="2" t="inlineStr">
+        <is>
+          <t>Mexico City</t>
+        </is>
+      </c>
+      <c r="G520" s="2" t="inlineStr">
+        <is>
+          <t>Ángel Zimbrón, Azcapotzalco</t>
+        </is>
+      </c>
+      <c r="H520" s="2" t="inlineStr">
+        <is>
+          <t>02099</t>
+        </is>
+      </c>
+      <c r="I520" s="2" t="inlineStr">
+        <is>
+          <t>https://www.basalmayoreo.com.mx</t>
+        </is>
+      </c>
+      <c r="J520" s="2" t="inlineStr"/>
+      <c r="K520" s="2" t="inlineStr"/>
+      <c r="L520" s="2" t="inlineStr"/>
+      <c r="M520" s="2" t="inlineStr"/>
+      <c r="N520" s="2" t="inlineStr">
+        <is>
+          <t>info@basalmayoreo.com.mx</t>
+        </is>
+      </c>
+      <c r="O520" s="2" t="inlineStr"/>
+      <c r="P520" s="2" t="inlineStr"/>
+      <c r="Q520" s="2" t="inlineStr"/>
+      <c r="R520" s="2" t="inlineStr"/>
+      <c r="S520" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/basalabarrotes/</t>
+        </is>
+      </c>
+      <c r="T520" s="2" t="inlineStr"/>
+      <c r="U520" s="2" t="inlineStr"/>
+      <c r="V520" s="2" t="inlineStr"/>
+      <c r="W520" s="2" t="inlineStr"/>
+      <c r="X520" s="2" t="inlineStr"/>
+      <c r="Y520" s="2" t="inlineStr"/>
+      <c r="Z520" s="2" t="inlineStr"/>
+      <c r="AA520" s="2" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>Comercial Vinícola</t>
+        </is>
+      </c>
+      <c r="B521" s="2" t="inlineStr"/>
+      <c r="C521" s="2" t="inlineStr">
+        <is>
+          <t>168591</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E521" s="2" t="inlineStr">
+        <is>
+          <t>Corregidora</t>
+        </is>
+      </c>
+      <c r="F521" s="2" t="inlineStr">
+        <is>
+          <t>Querétaro</t>
+        </is>
+      </c>
+      <c r="G521" s="2" t="inlineStr">
+        <is>
+          <t>Carretera Libre, de Celaya Km. 10</t>
+        </is>
+      </c>
+      <c r="H521" s="2" t="inlineStr">
+        <is>
+          <t>76900</t>
+        </is>
+      </c>
+      <c r="I521" s="2" t="inlineStr">
+        <is>
+          <t>https://www.comercialvinicola.com</t>
+        </is>
+      </c>
+      <c r="J521" s="2" t="inlineStr"/>
+      <c r="K521" s="2" t="inlineStr"/>
+      <c r="L521" s="2" t="inlineStr"/>
+      <c r="M521" s="2" t="inlineStr"/>
+      <c r="N521" s="2" t="inlineStr">
+        <is>
+          <t>ventas@comercialvinicola.com</t>
+        </is>
+      </c>
+      <c r="O521" s="2" t="inlineStr"/>
+      <c r="P521" s="2" t="inlineStr"/>
+      <c r="Q521" s="2" t="inlineStr"/>
+      <c r="R521" s="2" t="inlineStr"/>
+      <c r="S521" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/CVinicolaMX</t>
+        </is>
+      </c>
+      <c r="T521" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/cvinicolamx</t>
+        </is>
+      </c>
+      <c r="U521" s="2" t="inlineStr"/>
+      <c r="V521" s="2" t="inlineStr"/>
+      <c r="W521" s="2" t="inlineStr"/>
+      <c r="X521" s="2" t="inlineStr"/>
+      <c r="Y521" s="2" t="inlineStr"/>
+      <c r="Z521" s="2" t="inlineStr"/>
+      <c r="AA521" s="2" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>Bodegas Miró México</t>
+        </is>
+      </c>
+      <c r="B522" s="2" t="inlineStr"/>
+      <c r="C522" s="2" t="inlineStr">
+        <is>
+          <t>168590</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>Heroica Puebla de Zaragoza</t>
+        </is>
+      </c>
+      <c r="F522" s="2" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="G522" s="2" t="inlineStr">
+        <is>
+          <t>Rancho de La Rosa 1446, Xonaca</t>
+        </is>
+      </c>
+      <c r="H522" s="2" t="inlineStr">
+        <is>
+          <t>72370</t>
+        </is>
+      </c>
+      <c r="I522" s="2" t="inlineStr">
+        <is>
+          <t>https://bodegasmiro.com</t>
+        </is>
+      </c>
+      <c r="J522" s="2" t="inlineStr"/>
+      <c r="K522" s="2" t="inlineStr"/>
+      <c r="L522" s="2" t="inlineStr"/>
+      <c r="M522" s="2" t="inlineStr"/>
+      <c r="N522" s="2" t="inlineStr">
+        <is>
+          <t>info@bodegasmiro.com</t>
+        </is>
+      </c>
+      <c r="O522" s="2" t="inlineStr">
+        <is>
+          <t>+52 222 236 0008</t>
+        </is>
+      </c>
+      <c r="P522" s="2" t="inlineStr"/>
+      <c r="Q522" s="2" t="inlineStr"/>
+      <c r="R522" s="2" t="inlineStr"/>
+      <c r="S522" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/MiroBodegas/</t>
+        </is>
+      </c>
+      <c r="T522" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bodegasmiro/</t>
+        </is>
+      </c>
+      <c r="U522" s="2" t="inlineStr"/>
+      <c r="V522" s="2" t="inlineStr"/>
+      <c r="W522" s="2" t="inlineStr"/>
+      <c r="X522" s="2" t="inlineStr"/>
+      <c r="Y522" s="2" t="inlineStr"/>
+      <c r="Z522" s="2" t="inlineStr"/>
+      <c r="AA522" s="2" t="inlineStr"/>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>Mexital Gourmet</t>
+        </is>
+      </c>
+      <c r="B523" s="2" t="inlineStr"/>
+      <c r="C523" s="2" t="inlineStr">
+        <is>
+          <t>168589</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E523" s="2" t="inlineStr">
+        <is>
+          <t>Zapopan</t>
+        </is>
+      </c>
+      <c r="F523" s="2" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G523" s="2" t="inlineStr">
+        <is>
+          <t>Ludwig Van Beethoven 5133 B, Col. La Estancia</t>
+        </is>
+      </c>
+      <c r="H523" s="2" t="inlineStr">
+        <is>
+          <t>45030</t>
+        </is>
+      </c>
+      <c r="I523" s="2" t="inlineStr">
+        <is>
+          <t>https://mexitalgourmet.com</t>
+        </is>
+      </c>
+      <c r="J523" s="2" t="inlineStr"/>
+      <c r="K523" s="2" t="inlineStr"/>
+      <c r="L523" s="2" t="inlineStr"/>
+      <c r="M523" s="2" t="inlineStr"/>
+      <c r="N523" s="2" t="inlineStr">
+        <is>
+          <t>ventas@mexitalgourmet.com</t>
+        </is>
+      </c>
+      <c r="O523" s="2" t="inlineStr"/>
+      <c r="P523" s="2" t="inlineStr"/>
+      <c r="Q523" s="2" t="inlineStr"/>
+      <c r="R523" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/mexital-gourmet/</t>
+        </is>
+      </c>
+      <c r="S523" s="2" t="inlineStr"/>
+      <c r="T523" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mexital.gourmet/</t>
+        </is>
+      </c>
+      <c r="U523" s="2" t="inlineStr"/>
+      <c r="V523" s="2" t="inlineStr"/>
+      <c r="W523" s="2" t="inlineStr">
+        <is>
+          <t>Sebastian Baldassini</t>
+        </is>
+      </c>
+      <c r="X523" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="Y523" s="2" t="inlineStr"/>
+      <c r="Z523" s="2" t="inlineStr"/>
+      <c r="AA523" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/sebastian-baldassini-a27597b1</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>Alcohotel</t>
+        </is>
+      </c>
+      <c r="B524" s="2" t="inlineStr"/>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>168588</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>Cancún</t>
+        </is>
+      </c>
+      <c r="F524" s="2" t="inlineStr">
+        <is>
+          <t>Quintana Roo</t>
+        </is>
+      </c>
+      <c r="G524" s="2" t="inlineStr">
+        <is>
+          <t>Calle Insurgentes SM 307 MZA 266, Lote 1, Bodega 2</t>
+        </is>
+      </c>
+      <c r="H524" s="2" t="inlineStr">
+        <is>
+          <t>77560</t>
+        </is>
+      </c>
+      <c r="I524" s="2" t="inlineStr">
+        <is>
+          <t>https://www.alcohotel.com</t>
+        </is>
+      </c>
+      <c r="J524" s="2" t="inlineStr"/>
+      <c r="K524" s="2" t="inlineStr"/>
+      <c r="L524" s="2" t="inlineStr"/>
+      <c r="M524" s="2" t="inlineStr"/>
+      <c r="N524" s="2" t="inlineStr">
+        <is>
+          <t>ventas@alcohotel.com</t>
+        </is>
+      </c>
+      <c r="O524" s="2" t="inlineStr"/>
+      <c r="P524" s="2" t="inlineStr"/>
+      <c r="Q524" s="2" t="inlineStr"/>
+      <c r="R524" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/alcohotel/</t>
+        </is>
+      </c>
+      <c r="S524" s="2" t="inlineStr"/>
+      <c r="T524" s="2" t="inlineStr"/>
+      <c r="U524" s="2" t="inlineStr"/>
+      <c r="V524" s="2" t="inlineStr"/>
+      <c r="W524" s="2" t="inlineStr">
+        <is>
+          <t>Emilio De La Peña Hernandez</t>
+        </is>
+      </c>
+      <c r="X524" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CFO</t>
+        </is>
+      </c>
+      <c r="Y524" s="2" t="inlineStr"/>
+      <c r="Z524" s="2" t="inlineStr"/>
+      <c r="AA524" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/emilio-de-la-pe%C3%B1a-hernandez-029485192/</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>GB Almacenadora</t>
+        </is>
+      </c>
+      <c r="B525" s="2" t="inlineStr"/>
+      <c r="C525" s="2" t="inlineStr">
+        <is>
+          <t>168587</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E525" s="2" t="inlineStr">
+        <is>
+          <t>Iztapalapa</t>
+        </is>
+      </c>
+      <c r="F525" s="2" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="G525" s="2" t="inlineStr">
+        <is>
+          <t>Av. Transportistas 15, Bodega K13, Colonia Chinampac de Juárez</t>
+        </is>
+      </c>
+      <c r="H525" s="2" t="inlineStr">
+        <is>
+          <t>09208</t>
+        </is>
+      </c>
+      <c r="I525" s="2" t="inlineStr">
+        <is>
+          <t>https://gbalmacenadora.com</t>
+        </is>
+      </c>
+      <c r="J525" s="2" t="inlineStr"/>
+      <c r="K525" s="2" t="inlineStr"/>
+      <c r="L525" s="2" t="inlineStr"/>
+      <c r="M525" s="2" t="inlineStr"/>
+      <c r="N525" s="2" t="inlineStr">
+        <is>
+          <t>pedidos@gbalmacenadora.com</t>
+        </is>
+      </c>
+      <c r="O525" s="2" t="inlineStr">
+        <is>
+          <t>+52 998 626 7985</t>
+        </is>
+      </c>
+      <c r="P525" s="2" t="inlineStr"/>
+      <c r="Q525" s="2" t="inlineStr"/>
+      <c r="R525" s="2" t="inlineStr"/>
+      <c r="S525" s="2" t="inlineStr"/>
+      <c r="T525" s="2" t="inlineStr"/>
+      <c r="U525" s="2" t="inlineStr"/>
+      <c r="V525" s="2" t="inlineStr"/>
+      <c r="W525" s="2" t="inlineStr">
+        <is>
+          <t>Javier Martin</t>
+        </is>
+      </c>
+      <c r="X525" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="Y525" s="2" t="inlineStr"/>
+      <c r="Z525" s="2" t="inlineStr"/>
+      <c r="AA525" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/javier-martin-04798899/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>